<commit_message>
update readme and repo dependencies
</commit_message>
<xml_diff>
--- a/Local/Data/Export/DQ-Report_meDIC_StandortName_FHIR_2020.xlsx
+++ b/Local/Data/Export/DQ-Report_meDIC_StandortName_FHIR_2020.xlsx
@@ -8,12 +8,13 @@
   <sheets>
     <sheet name="DQ_Metrics" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="DQ_Violations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Semantics" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="150">
   <si>
     <t xml:space="preserve">Abbreviation</t>
   </si>
@@ -111,21 +112,21 @@
     <t xml:space="preserve">RD Case Dissimilarity Rate</t>
   </si>
   <si>
+    <t xml:space="preserve">aPatient</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyzed Patients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45</t>
+  </si>
+  <si>
     <t xml:space="preserve">aCase</t>
   </si>
   <si>
     <t xml:space="preserve">Analyzed Cases</t>
   </si>
   <si>
-    <t xml:space="preserve">45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aPatient</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analyzed Patients</t>
-  </si>
-  <si>
     <t xml:space="preserve">im_misg</t>
   </si>
   <si>
@@ -240,7 +241,7 @@
     <t xml:space="preserve">Execution Time</t>
   </si>
   <si>
-    <t xml:space="preserve">0.06</t>
+    <t xml:space="preserve">0.05</t>
   </si>
   <si>
     <t xml:space="preserve">par_computing</t>
@@ -318,7 +319,7 @@
     <t xml:space="preserve">E84.0</t>
   </si>
   <si>
-    <t xml:space="preserve">Missing Orpha Code.  </t>
+    <t xml:space="preserve">Missing Orpha Code.  Missing Orpha Code.  </t>
   </si>
   <si>
     <t xml:space="preserve">E84.1</t>
@@ -399,7 +400,70 @@
     <t xml:space="preserve">Ambiguous Orphacoding. ICD10-Orpha combination: E03.1 - 442 is implausible according to Alpha-ID-SE. </t>
   </si>
   <si>
-    <t xml:space="preserve">Following items are missing:  Kontakt_Klasse , Fall_Status , DiagnoseRolle</t>
+    <t xml:space="preserve">Following data items are missing:  Kontakt_Klasse , Fall_Status , DiagnoseRolle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short_Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completeness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator assesses the metadata completeness. Further details and examples are available under DOI:10.1055/a-2006-1018.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator assesses the data completeness of a given data set. The publication DOI:10.1055/a-2006-1018 provides more details and examples.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plausibility</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator assesses the plausibility of selected data values regarding outliers. The publication DOI:10.1055/a-2006-1018 provides more details and examples.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dqi_pl_spr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semantic Plausibility Rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator assesses the plausibility of selected data values regarding semantic contradictions. The publication DOI:10.1055/a-2006-1018 provides more details and examples.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dqi_co_scr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subject Completeness Rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator assesses the completeness of subject records. Further details and examples can be found under DOI:10.1055/a-2006-1018.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dqi_co_ccr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Case Completeness Rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator assesses the completeness of data values required for recording the case module in a given data set. Further details and examples are available under DOI:10.1055/a-2006-1018.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator assesses whether all cases with tracer diagnoses (icd_tracer) are coded using Orphacodes. Further details and examples are available under DOI:10.1055/a-2006-1018.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator assesses the semantic plausibility of coded RD diagnoses according to the standard terminology Alpha-ID-SE. The publication DOI:10.1055/a-2006-1018 provides more details and examples.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uniquness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator assesses the semantic uniqueness of RD diagnoses in a given data set. More details are available in the publication DOI:10.1055/a-2006-1018.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This indicator assesses the syntactic uniqueness of RD diagnoses in a given data set. Further details and examples are available in the publication DOI:10.1055/a-2006-1018.</t>
   </si>
 </sst>
 </file>
@@ -738,6 +802,33 @@
     <col min="1" max="1" width="14.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="60.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="9.15" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="9.15" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="9.15" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="9.15" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="9.15" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="9.15" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="9.15" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="9.15" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="9.15" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="9.15" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="9.15" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="9.15" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="9.15" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="9.15" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="9.15" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="9.15" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="9.15" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="9.15" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="9.15" hidden="0" customWidth="1"/>
+    <col min="23" max="23" width="9.15" hidden="0" customWidth="1"/>
+    <col min="24" max="24" width="9.15" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="9.15" hidden="0" customWidth="1"/>
+    <col min="26" max="26" width="9.15" hidden="0" customWidth="1"/>
+    <col min="27" max="27" width="9.15" hidden="0" customWidth="1"/>
+    <col min="28" max="28" width="9.15" hidden="0" customWidth="1"/>
+    <col min="29" max="29" width="9.15" hidden="0" customWidth="1"/>
+    <col min="30" max="30" width="9.15" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1117,6 +1208,31 @@
     <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="9.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="101.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="9.15" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="9.15" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="9.15" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="9.15" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="9.15" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="9.15" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="9.15" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="9.15" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="9.15" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="9.15" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="9.15" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="9.15" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="9.15" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="9.15" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="9.15" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="9.15" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="9.15" hidden="0" customWidth="1"/>
+    <col min="23" max="23" width="9.15" hidden="0" customWidth="1"/>
+    <col min="24" max="24" width="9.15" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="9.15" hidden="0" customWidth="1"/>
+    <col min="26" max="26" width="9.15" hidden="0" customWidth="1"/>
+    <col min="27" max="27" width="9.15" hidden="0" customWidth="1"/>
+    <col min="28" max="28" width="9.15" hidden="0" customWidth="1"/>
+    <col min="29" max="29" width="9.15" hidden="0" customWidth="1"/>
+    <col min="30" max="30" width="9.15" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1292,4 +1408,201 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="12.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="29.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="12.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="198.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="9.15" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="9.15" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="9.15" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="9.15" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="9.15" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="9.15" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="9.15" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="9.15" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="9.15" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="9.15" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="9.15" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="9.15" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="9.15" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="9.15" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="9.15" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="9.15" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="9.15" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="9.15" hidden="0" customWidth="1"/>
+    <col min="23" max="23" width="9.15" hidden="0" customWidth="1"/>
+    <col min="24" max="24" width="9.15" hidden="0" customWidth="1"/>
+    <col min="25" max="25" width="9.15" hidden="0" customWidth="1"/>
+    <col min="26" max="26" width="9.15" hidden="0" customWidth="1"/>
+    <col min="27" max="27" width="9.15" hidden="0" customWidth="1"/>
+    <col min="28" max="28" width="9.15" hidden="0" customWidth="1"/>
+    <col min="29" max="29" width="9.15" hidden="0" customWidth="1"/>
+    <col min="30" max="30" width="9.15" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>134</v>
+      </c>
+      <c r="D4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>142</v>
+      </c>
+      <c r="B7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>131</v>
+      </c>
+      <c r="D8" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>134</v>
+      </c>
+      <c r="D9" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>147</v>
+      </c>
+      <c r="D10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D11" t="s">
+        <v>149</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>